<commit_message>
update payload for user import
</commit_message>
<xml_diff>
--- a/sample-format/userPasswordUpdate (2).xlsx
+++ b/sample-format/userPasswordUpdate (2).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\deskTop\WHO-lepo\March-2024-population_user_Password_update\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\gitHub_source_code\excel_to_Json_Converter_angularJS\sample-format\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D3C60FE-BD58-400E-8C4F-A5F7DAE8DC6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F55DDB0-FA26-449B-8D8E-98D61E72EDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4717,6 +4717,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010064994C001712374395B345EB88ED991F" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8c1a62579524e26006c6d5335831b55c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f9770305-a86c-4dd4-a8e3-5283c3e6bf99" xmlns:ns3="3f48127a-ff27-4c8f-88c3-e54b29f41588" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="658091719f3253a39288b5ed2add5a7b" ns2:_="" ns3:_="">
     <xsd:import namespace="f9770305-a86c-4dd4-a8e3-5283c3e6bf99"/>
@@ -4913,22 +4928,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18A4371F-7DC5-4CF4-A869-E47776CCD6EB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACBAC26C-ABD4-4796-8551-545E34A88729}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E76993AC-6818-4630-B1D6-F654BE5E03B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4945,21 +4962,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACBAC26C-ABD4-4796-8551-545E34A88729}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18A4371F-7DC5-4CF4-A869-E47776CCD6EB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>